<commit_message>
Update on AGE-2 SP
</commit_message>
<xml_diff>
--- a/excel_data/gcg_cardlist_hk.xlsx
+++ b/excel_data/gcg_cardlist_hk.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FLC\Desktop\JavaScript\Gundam Card Web\gundam-card-web\excel_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F507551-9ADF-4231-AD45-FEF45B651A8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9695A08-133C-4915-B744-049A01BFDD6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8174,9 +8174,6 @@
     <t>GD05-024</t>
   </si>
   <si>
-    <t>高達AGE-1 普通型(特別配色)</t>
-  </si>
-  <si>
     <t>【破壞時】選擇我方廢棄區中1張綠色的〔地球聯邦〕機師卡牌。將其加入手牌。若那樣做的話，則丟棄我方的1張手牌。</t>
   </si>
   <si>
@@ -9250,6 +9247,32 @@
   </si>
   <si>
     <t>特徴〔預防者〕 / 「露洛莉亞・奈」</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>高達AGE-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="新細明體"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 普通型(特別配色)</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -9257,7 +9280,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -9271,6 +9294,13 @@
       <family val="3"/>
       <charset val="136"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="2"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="2">
@@ -47327,7 +47357,7 @@
         <v>2498</v>
       </c>
     </row>
-    <row r="858" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="858" spans="1:14" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A858" t="s">
         <v>2562</v>
       </c>
@@ -47335,7 +47365,7 @@
         <v>50</v>
       </c>
       <c r="C858" t="s">
-        <v>2563</v>
+        <v>2894</v>
       </c>
       <c r="D858" t="s">
         <v>19</v>
@@ -47350,7 +47380,7 @@
         <v>21</v>
       </c>
       <c r="H858" t="s">
-        <v>2564</v>
+        <v>2563</v>
       </c>
       <c r="I858" t="s">
         <v>23</v>
@@ -47373,13 +47403,13 @@
     </row>
     <row r="859" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A859" t="s">
-        <v>2565</v>
+        <v>2564</v>
       </c>
       <c r="B859" t="s">
         <v>50</v>
       </c>
       <c r="C859" t="s">
-        <v>2566</v>
+        <v>2565</v>
       </c>
       <c r="D859" t="s">
         <v>26</v>
@@ -47394,7 +47424,7 @@
         <v>21</v>
       </c>
       <c r="H859" t="s">
-        <v>2567</v>
+        <v>2566</v>
       </c>
       <c r="I859" t="s">
         <v>23</v>
@@ -47417,7 +47447,7 @@
     </row>
     <row r="860" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A860" t="s">
-        <v>2568</v>
+        <v>2567</v>
       </c>
       <c r="B860" t="s">
         <v>50</v>
@@ -47438,16 +47468,16 @@
         <v>21</v>
       </c>
       <c r="H860" t="s">
-        <v>2569</v>
+        <v>2568</v>
       </c>
       <c r="I860" t="s">
         <v>23</v>
       </c>
       <c r="J860" t="s">
+        <v>2569</v>
+      </c>
+      <c r="K860" t="s">
         <v>2570</v>
-      </c>
-      <c r="K860" t="s">
-        <v>2571</v>
       </c>
       <c r="L860" t="s">
         <v>44</v>
@@ -47461,7 +47491,7 @@
     </row>
     <row r="861" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A861" t="s">
-        <v>2572</v>
+        <v>2571</v>
       </c>
       <c r="B861" t="s">
         <v>68</v>
@@ -47505,13 +47535,13 @@
     </row>
     <row r="862" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A862" t="s">
-        <v>2573</v>
+        <v>2572</v>
       </c>
       <c r="B862" t="s">
         <v>68</v>
       </c>
       <c r="C862" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
       <c r="D862" t="s">
         <v>44</v>
@@ -47526,7 +47556,7 @@
         <v>21</v>
       </c>
       <c r="H862" t="s">
-        <v>2575</v>
+        <v>2574</v>
       </c>
       <c r="I862" t="s">
         <v>23</v>
@@ -47535,7 +47565,7 @@
         <v>2544</v>
       </c>
       <c r="K862" t="s">
-        <v>2576</v>
+        <v>2575</v>
       </c>
       <c r="L862" t="s">
         <v>66</v>
@@ -47549,13 +47579,13 @@
     </row>
     <row r="863" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A863" t="s">
-        <v>2577</v>
+        <v>2576</v>
       </c>
       <c r="B863" t="s">
         <v>68</v>
       </c>
       <c r="C863" t="s">
-        <v>2578</v>
+        <v>2577</v>
       </c>
       <c r="D863" t="s">
         <v>44</v>
@@ -47579,7 +47609,7 @@
         <v>2544</v>
       </c>
       <c r="K863" t="s">
-        <v>2576</v>
+        <v>2575</v>
       </c>
       <c r="L863" t="s">
         <v>44</v>
@@ -47593,7 +47623,7 @@
     </row>
     <row r="864" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A864" t="s">
-        <v>2579</v>
+        <v>2578</v>
       </c>
       <c r="B864" t="s">
         <v>68</v>
@@ -47614,7 +47644,7 @@
         <v>21</v>
       </c>
       <c r="H864" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="I864" t="s">
         <v>23</v>
@@ -47623,7 +47653,7 @@
         <v>548</v>
       </c>
       <c r="K864" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="L864" t="s">
         <v>44</v>
@@ -47637,7 +47667,7 @@
     </row>
     <row r="865" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A865" t="s">
-        <v>2582</v>
+        <v>2581</v>
       </c>
       <c r="B865" t="s">
         <v>68</v>
@@ -47681,13 +47711,13 @@
     </row>
     <row r="866" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A866" t="s">
-        <v>2583</v>
+        <v>2582</v>
       </c>
       <c r="B866" t="s">
         <v>68</v>
       </c>
       <c r="C866" t="s">
-        <v>2584</v>
+        <v>2583</v>
       </c>
       <c r="D866" t="s">
         <v>26</v>
@@ -47708,10 +47738,10 @@
         <v>23</v>
       </c>
       <c r="J866" t="s">
+        <v>2584</v>
+      </c>
+      <c r="K866" t="s">
         <v>2585</v>
-      </c>
-      <c r="K866" t="s">
-        <v>2586</v>
       </c>
       <c r="L866" t="s">
         <v>26</v>
@@ -47725,13 +47755,13 @@
     </row>
     <row r="867" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A867" t="s">
-        <v>2587</v>
+        <v>2586</v>
       </c>
       <c r="B867" t="s">
         <v>16</v>
       </c>
       <c r="C867" t="s">
-        <v>2588</v>
+        <v>2587</v>
       </c>
       <c r="D867" t="s">
         <v>31</v>
@@ -47746,16 +47776,16 @@
         <v>21</v>
       </c>
       <c r="H867" t="s">
-        <v>2589</v>
+        <v>2588</v>
       </c>
       <c r="I867" t="s">
         <v>23</v>
       </c>
       <c r="J867" t="s">
+        <v>2589</v>
+      </c>
+      <c r="K867" t="s">
         <v>2590</v>
-      </c>
-      <c r="K867" t="s">
-        <v>2591</v>
       </c>
       <c r="L867" t="s">
         <v>19</v>
@@ -47769,13 +47799,13 @@
     </row>
     <row r="868" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A868" t="s">
-        <v>2592</v>
+        <v>2591</v>
       </c>
       <c r="B868" t="s">
         <v>16</v>
       </c>
       <c r="C868" t="s">
-        <v>2593</v>
+        <v>2592</v>
       </c>
       <c r="D868" t="s">
         <v>44</v>
@@ -47790,16 +47820,16 @@
         <v>21</v>
       </c>
       <c r="H868" t="s">
-        <v>2594</v>
+        <v>2593</v>
       </c>
       <c r="I868" t="s">
         <v>23</v>
       </c>
       <c r="J868" t="s">
+        <v>2594</v>
+      </c>
+      <c r="K868" t="s">
         <v>2595</v>
-      </c>
-      <c r="K868" t="s">
-        <v>2596</v>
       </c>
       <c r="L868" t="s">
         <v>44</v>
@@ -47813,13 +47843,13 @@
     </row>
     <row r="869" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A869" t="s">
-        <v>2597</v>
+        <v>2596</v>
       </c>
       <c r="B869" t="s">
         <v>35</v>
       </c>
       <c r="C869" t="s">
-        <v>2598</v>
+        <v>2597</v>
       </c>
       <c r="D869" t="s">
         <v>19</v>
@@ -47834,16 +47864,16 @@
         <v>21</v>
       </c>
       <c r="H869" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="I869" t="s">
         <v>23</v>
       </c>
       <c r="J869" t="s">
+        <v>2599</v>
+      </c>
+      <c r="K869" t="s">
         <v>2600</v>
-      </c>
-      <c r="K869" t="s">
-        <v>2601</v>
       </c>
       <c r="L869" t="s">
         <v>26</v>
@@ -47857,13 +47887,13 @@
     </row>
     <row r="870" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A870" t="s">
-        <v>2602</v>
+        <v>2601</v>
       </c>
       <c r="B870" t="s">
         <v>35</v>
       </c>
       <c r="C870" t="s">
-        <v>2603</v>
+        <v>2602</v>
       </c>
       <c r="D870" t="s">
         <v>18</v>
@@ -47878,16 +47908,16 @@
         <v>21</v>
       </c>
       <c r="H870" t="s">
-        <v>2604</v>
+        <v>2603</v>
       </c>
       <c r="I870" t="s">
         <v>23</v>
       </c>
       <c r="J870" t="s">
-        <v>2605</v>
+        <v>2604</v>
       </c>
       <c r="K870" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="L870" t="s">
         <v>26</v>
@@ -47901,13 +47931,13 @@
     </row>
     <row r="871" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A871" t="s">
-        <v>2606</v>
+        <v>2605</v>
       </c>
       <c r="B871" t="s">
         <v>35</v>
       </c>
       <c r="C871" t="s">
-        <v>2607</v>
+        <v>2606</v>
       </c>
       <c r="D871" t="s">
         <v>1704</v>
@@ -47922,13 +47952,13 @@
         <v>21</v>
       </c>
       <c r="H871" t="s">
-        <v>2608</v>
+        <v>2607</v>
       </c>
       <c r="I871" t="s">
         <v>23</v>
       </c>
       <c r="J871" t="s">
-        <v>2595</v>
+        <v>2594</v>
       </c>
       <c r="K871" t="s">
         <v>775</v>
@@ -47945,13 +47975,13 @@
     </row>
     <row r="872" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A872" t="s">
-        <v>2609</v>
+        <v>2608</v>
       </c>
       <c r="B872" t="s">
         <v>35</v>
       </c>
       <c r="C872" t="s">
-        <v>2610</v>
+        <v>2609</v>
       </c>
       <c r="D872" t="s">
         <v>31</v>
@@ -47966,7 +47996,7 @@
         <v>21</v>
       </c>
       <c r="H872" t="s">
-        <v>2611</v>
+        <v>2610</v>
       </c>
       <c r="I872" t="s">
         <v>23</v>
@@ -47989,13 +48019,13 @@
     </row>
     <row r="873" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A873" t="s">
-        <v>2612</v>
+        <v>2611</v>
       </c>
       <c r="B873" t="s">
         <v>50</v>
       </c>
       <c r="C873" t="s">
-        <v>2613</v>
+        <v>2612</v>
       </c>
       <c r="D873" t="s">
         <v>44</v>
@@ -48010,16 +48040,16 @@
         <v>21</v>
       </c>
       <c r="H873" t="s">
-        <v>2614</v>
+        <v>2613</v>
       </c>
       <c r="I873" t="s">
         <v>23</v>
       </c>
       <c r="J873" t="s">
-        <v>2595</v>
+        <v>2594</v>
       </c>
       <c r="K873" t="s">
-        <v>2615</v>
+        <v>2614</v>
       </c>
       <c r="L873" t="s">
         <v>26</v>
@@ -48033,13 +48063,13 @@
     </row>
     <row r="874" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A874" t="s">
-        <v>2616</v>
+        <v>2615</v>
       </c>
       <c r="B874" t="s">
         <v>50</v>
       </c>
       <c r="C874" t="s">
-        <v>2617</v>
+        <v>2616</v>
       </c>
       <c r="D874" t="s">
         <v>44</v>
@@ -48060,10 +48090,10 @@
         <v>23</v>
       </c>
       <c r="J874" t="s">
-        <v>2595</v>
+        <v>2594</v>
       </c>
       <c r="K874" t="s">
-        <v>2618</v>
+        <v>2617</v>
       </c>
       <c r="L874" t="s">
         <v>66</v>
@@ -48077,13 +48107,13 @@
     </row>
     <row r="875" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A875" t="s">
-        <v>2619</v>
+        <v>2618</v>
       </c>
       <c r="B875" t="s">
         <v>50</v>
       </c>
       <c r="C875" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="D875" t="s">
         <v>26</v>
@@ -48098,16 +48128,16 @@
         <v>21</v>
       </c>
       <c r="H875" t="s">
-        <v>2621</v>
+        <v>2620</v>
       </c>
       <c r="I875" t="s">
         <v>23</v>
       </c>
       <c r="J875" t="s">
+        <v>2594</v>
+      </c>
+      <c r="K875" t="s">
         <v>2595</v>
-      </c>
-      <c r="K875" t="s">
-        <v>2596</v>
       </c>
       <c r="L875" t="s">
         <v>26</v>
@@ -48121,13 +48151,13 @@
     </row>
     <row r="876" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A876" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
       <c r="B876" t="s">
         <v>68</v>
       </c>
       <c r="C876" t="s">
-        <v>2623</v>
+        <v>2622</v>
       </c>
       <c r="D876" t="s">
         <v>66</v>
@@ -48148,7 +48178,7 @@
         <v>23</v>
       </c>
       <c r="J876" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
       <c r="K876" t="s">
         <v>55</v>
@@ -48165,13 +48195,13 @@
     </row>
     <row r="877" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A877" t="s">
-        <v>2624</v>
+        <v>2623</v>
       </c>
       <c r="B877" t="s">
         <v>68</v>
       </c>
       <c r="C877" t="s">
-        <v>2625</v>
+        <v>2624</v>
       </c>
       <c r="D877" t="s">
         <v>66</v>
@@ -48192,7 +48222,7 @@
         <v>23</v>
       </c>
       <c r="J877" t="s">
-        <v>2605</v>
+        <v>2604</v>
       </c>
       <c r="K877" t="s">
         <v>55</v>
@@ -48209,13 +48239,13 @@
     </row>
     <row r="878" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A878" t="s">
-        <v>2626</v>
+        <v>2625</v>
       </c>
       <c r="B878" t="s">
         <v>68</v>
       </c>
       <c r="C878" t="s">
-        <v>2627</v>
+        <v>2626</v>
       </c>
       <c r="D878" t="s">
         <v>44</v>
@@ -48230,16 +48260,16 @@
         <v>21</v>
       </c>
       <c r="H878" t="s">
-        <v>2628</v>
+        <v>2627</v>
       </c>
       <c r="I878" t="s">
         <v>23</v>
       </c>
       <c r="J878" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
       <c r="K878" t="s">
-        <v>2629</v>
+        <v>2628</v>
       </c>
       <c r="L878" t="s">
         <v>44</v>
@@ -48253,13 +48283,13 @@
     </row>
     <row r="879" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A879" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
       <c r="B879" t="s">
         <v>68</v>
       </c>
       <c r="C879" t="s">
-        <v>2631</v>
+        <v>2630</v>
       </c>
       <c r="D879" t="s">
         <v>26</v>
@@ -48274,16 +48304,16 @@
         <v>21</v>
       </c>
       <c r="H879" t="s">
-        <v>2632</v>
+        <v>2631</v>
       </c>
       <c r="I879" t="s">
         <v>23</v>
       </c>
       <c r="J879" t="s">
-        <v>2595</v>
+        <v>2594</v>
       </c>
       <c r="K879" t="s">
-        <v>2615</v>
+        <v>2614</v>
       </c>
       <c r="L879" t="s">
         <v>44</v>
@@ -48297,13 +48327,13 @@
     </row>
     <row r="880" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A880" t="s">
-        <v>2633</v>
+        <v>2632</v>
       </c>
       <c r="B880" t="s">
         <v>68</v>
       </c>
       <c r="C880" t="s">
-        <v>2634</v>
+        <v>2633</v>
       </c>
       <c r="D880" t="s">
         <v>26</v>
@@ -48318,16 +48348,16 @@
         <v>21</v>
       </c>
       <c r="H880" t="s">
-        <v>2635</v>
+        <v>2634</v>
       </c>
       <c r="I880" t="s">
         <v>80</v>
       </c>
       <c r="J880" t="s">
-        <v>2595</v>
+        <v>2594</v>
       </c>
       <c r="K880" t="s">
-        <v>2618</v>
+        <v>2617</v>
       </c>
       <c r="L880" t="s">
         <v>44</v>
@@ -48341,13 +48371,13 @@
     </row>
     <row r="881" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A881" t="s">
-        <v>2636</v>
+        <v>2635</v>
       </c>
       <c r="B881" t="s">
         <v>68</v>
       </c>
       <c r="C881" t="s">
-        <v>2637</v>
+        <v>2636</v>
       </c>
       <c r="D881" t="s">
         <v>44</v>
@@ -48368,7 +48398,7 @@
         <v>38</v>
       </c>
       <c r="J881" t="s">
-        <v>2595</v>
+        <v>2594</v>
       </c>
       <c r="K881" t="s">
         <v>553</v>
@@ -48385,7 +48415,7 @@
     </row>
     <row r="882" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A882" t="s">
-        <v>2638</v>
+        <v>2637</v>
       </c>
       <c r="B882" t="s">
         <v>68</v>
@@ -48406,7 +48436,7 @@
         <v>21</v>
       </c>
       <c r="H882" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="I882" t="s">
         <v>23</v>
@@ -48429,13 +48459,13 @@
     </row>
     <row r="883" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A883" t="s">
-        <v>2639</v>
+        <v>2638</v>
       </c>
       <c r="B883" t="s">
         <v>16</v>
       </c>
       <c r="C883" t="s">
-        <v>2640</v>
+        <v>2639</v>
       </c>
       <c r="D883" t="s">
         <v>31</v>
@@ -48450,7 +48480,7 @@
         <v>21</v>
       </c>
       <c r="H883" t="s">
-        <v>2641</v>
+        <v>2640</v>
       </c>
       <c r="I883" t="s">
         <v>23</v>
@@ -48473,13 +48503,13 @@
     </row>
     <row r="884" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A884" t="s">
-        <v>2642</v>
+        <v>2641</v>
       </c>
       <c r="B884" t="s">
         <v>16</v>
       </c>
       <c r="C884" t="s">
-        <v>2643</v>
+        <v>2642</v>
       </c>
       <c r="D884" t="s">
         <v>66</v>
@@ -48494,7 +48524,7 @@
         <v>21</v>
       </c>
       <c r="H884" t="s">
-        <v>2644</v>
+        <v>2643</v>
       </c>
       <c r="I884" t="s">
         <v>23</v>
@@ -48517,13 +48547,13 @@
     </row>
     <row r="885" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A885" t="s">
-        <v>2645</v>
+        <v>2644</v>
       </c>
       <c r="B885" t="s">
         <v>16</v>
       </c>
       <c r="C885" t="s">
-        <v>2646</v>
+        <v>2645</v>
       </c>
       <c r="D885" t="s">
         <v>31</v>
@@ -48538,7 +48568,7 @@
         <v>21</v>
       </c>
       <c r="H885" t="s">
-        <v>2647</v>
+        <v>2646</v>
       </c>
       <c r="I885" t="s">
         <v>23</v>
@@ -48561,13 +48591,13 @@
     </row>
     <row r="886" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A886" t="s">
-        <v>2648</v>
+        <v>2647</v>
       </c>
       <c r="B886" t="s">
         <v>35</v>
       </c>
       <c r="C886" t="s">
-        <v>2640</v>
+        <v>2639</v>
       </c>
       <c r="D886" t="s">
         <v>19</v>
@@ -48582,7 +48612,7 @@
         <v>21</v>
       </c>
       <c r="H886" t="s">
-        <v>2649</v>
+        <v>2648</v>
       </c>
       <c r="I886" t="s">
         <v>23</v>
@@ -48605,13 +48635,13 @@
     </row>
     <row r="887" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A887" t="s">
-        <v>2650</v>
+        <v>2649</v>
       </c>
       <c r="B887" t="s">
         <v>35</v>
       </c>
       <c r="C887" t="s">
-        <v>2651</v>
+        <v>2650</v>
       </c>
       <c r="D887" t="s">
         <v>44</v>
@@ -48626,7 +48656,7 @@
         <v>21</v>
       </c>
       <c r="H887" t="s">
-        <v>2652</v>
+        <v>2651</v>
       </c>
       <c r="I887" t="s">
         <v>23</v>
@@ -48635,7 +48665,7 @@
         <v>475</v>
       </c>
       <c r="K887" t="s">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="L887" t="s">
         <v>44</v>
@@ -48649,13 +48679,13 @@
     </row>
     <row r="888" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A888" t="s">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="B888" t="s">
         <v>35</v>
       </c>
       <c r="C888" t="s">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="D888" t="s">
         <v>30</v>
@@ -48670,7 +48700,7 @@
         <v>21</v>
       </c>
       <c r="H888" t="s">
-        <v>2656</v>
+        <v>2655</v>
       </c>
       <c r="I888" t="s">
         <v>38</v>
@@ -48679,7 +48709,7 @@
         <v>475</v>
       </c>
       <c r="K888" t="s">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="L888" t="s">
         <v>18</v>
@@ -48693,7 +48723,7 @@
     </row>
     <row r="889" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A889" t="s">
-        <v>2657</v>
+        <v>2656</v>
       </c>
       <c r="B889" t="s">
         <v>35</v>
@@ -48714,7 +48744,7 @@
         <v>21</v>
       </c>
       <c r="H889" t="s">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="I889" t="s">
         <v>23</v>
@@ -48737,13 +48767,13 @@
     </row>
     <row r="890" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A890" t="s">
-        <v>2659</v>
+        <v>2658</v>
       </c>
       <c r="B890" t="s">
         <v>50</v>
       </c>
       <c r="C890" t="s">
-        <v>2660</v>
+        <v>2659</v>
       </c>
       <c r="D890" t="s">
         <v>26</v>
@@ -48781,13 +48811,13 @@
     </row>
     <row r="891" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A891" t="s">
-        <v>2661</v>
+        <v>2660</v>
       </c>
       <c r="B891" t="s">
         <v>50</v>
       </c>
       <c r="C891" t="s">
-        <v>2662</v>
+        <v>2661</v>
       </c>
       <c r="D891" t="s">
         <v>26</v>
@@ -48802,7 +48832,7 @@
         <v>21</v>
       </c>
       <c r="H891" t="s">
-        <v>2663</v>
+        <v>2662</v>
       </c>
       <c r="I891" t="s">
         <v>23</v>
@@ -48811,7 +48841,7 @@
         <v>475</v>
       </c>
       <c r="K891" t="s">
-        <v>2664</v>
+        <v>2663</v>
       </c>
       <c r="L891" t="s">
         <v>26</v>
@@ -48825,13 +48855,13 @@
     </row>
     <row r="892" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A892" t="s">
-        <v>2665</v>
+        <v>2664</v>
       </c>
       <c r="B892" t="s">
         <v>50</v>
       </c>
       <c r="C892" t="s">
-        <v>2666</v>
+        <v>2665</v>
       </c>
       <c r="D892" t="s">
         <v>26</v>
@@ -48869,7 +48899,7 @@
     </row>
     <row r="893" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A893" t="s">
-        <v>2667</v>
+        <v>2666</v>
       </c>
       <c r="B893" t="s">
         <v>50</v>
@@ -48890,7 +48920,7 @@
         <v>21</v>
       </c>
       <c r="H893" t="s">
-        <v>2668</v>
+        <v>2667</v>
       </c>
       <c r="I893" t="s">
         <v>23</v>
@@ -48913,13 +48943,13 @@
     </row>
     <row r="894" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A894" t="s">
-        <v>2669</v>
+        <v>2668</v>
       </c>
       <c r="B894" t="s">
         <v>50</v>
       </c>
       <c r="C894" t="s">
-        <v>2670</v>
+        <v>2669</v>
       </c>
       <c r="D894" t="s">
         <v>19</v>
@@ -48934,7 +48964,7 @@
         <v>21</v>
       </c>
       <c r="H894" t="s">
-        <v>2671</v>
+        <v>2670</v>
       </c>
       <c r="I894" t="s">
         <v>23</v>
@@ -48957,13 +48987,13 @@
     </row>
     <row r="895" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A895" t="s">
-        <v>2672</v>
+        <v>2671</v>
       </c>
       <c r="B895" t="s">
         <v>68</v>
       </c>
       <c r="C895" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="D895" t="s">
         <v>66</v>
@@ -48978,7 +49008,7 @@
         <v>21</v>
       </c>
       <c r="H895" t="s">
-        <v>2674</v>
+        <v>2673</v>
       </c>
       <c r="I895" t="s">
         <v>23</v>
@@ -49001,13 +49031,13 @@
     </row>
     <row r="896" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A896" t="s">
-        <v>2675</v>
+        <v>2674</v>
       </c>
       <c r="B896" t="s">
         <v>68</v>
       </c>
       <c r="C896" t="s">
-        <v>2676</v>
+        <v>2675</v>
       </c>
       <c r="D896" t="s">
         <v>66</v>
@@ -49045,13 +49075,13 @@
     </row>
     <row r="897" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A897" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
       <c r="B897" t="s">
         <v>68</v>
       </c>
       <c r="C897" t="s">
-        <v>2662</v>
+        <v>2661</v>
       </c>
       <c r="D897" t="s">
         <v>44</v>
@@ -49089,7 +49119,7 @@
     </row>
     <row r="898" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A898" t="s">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="B898" t="s">
         <v>68</v>
@@ -49110,7 +49140,7 @@
         <v>21</v>
       </c>
       <c r="H898" t="s">
-        <v>2679</v>
+        <v>2678</v>
       </c>
       <c r="I898" t="s">
         <v>23</v>
@@ -49119,7 +49149,7 @@
         <v>1757</v>
       </c>
       <c r="K898" t="s">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="L898" t="s">
         <v>44</v>
@@ -49133,13 +49163,13 @@
     </row>
     <row r="899" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A899" t="s">
-        <v>2681</v>
+        <v>2680</v>
       </c>
       <c r="B899" t="s">
         <v>68</v>
       </c>
       <c r="C899" t="s">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="D899" t="s">
         <v>66</v>
@@ -49154,7 +49184,7 @@
         <v>21</v>
       </c>
       <c r="H899" t="s">
-        <v>2683</v>
+        <v>2682</v>
       </c>
       <c r="I899" t="s">
         <v>23</v>
@@ -49177,13 +49207,13 @@
     </row>
     <row r="900" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A900" t="s">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="B900" t="s">
         <v>16</v>
       </c>
       <c r="C900" t="s">
-        <v>2623</v>
+        <v>2622</v>
       </c>
       <c r="D900" t="s">
         <v>26</v>
@@ -49198,16 +49228,16 @@
         <v>21</v>
       </c>
       <c r="H900" t="s">
-        <v>2685</v>
+        <v>2684</v>
       </c>
       <c r="I900" t="s">
         <v>23</v>
       </c>
       <c r="J900" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
       <c r="K900" t="s">
-        <v>2686</v>
+        <v>2685</v>
       </c>
       <c r="L900" t="s">
         <v>44</v>
@@ -49221,13 +49251,13 @@
     </row>
     <row r="901" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A901" t="s">
-        <v>2687</v>
+        <v>2686</v>
       </c>
       <c r="B901" t="s">
         <v>16</v>
       </c>
       <c r="C901" t="s">
-        <v>2688</v>
+        <v>2687</v>
       </c>
       <c r="D901" t="s">
         <v>18</v>
@@ -49242,7 +49272,7 @@
         <v>21</v>
       </c>
       <c r="H901" t="s">
-        <v>2689</v>
+        <v>2688</v>
       </c>
       <c r="I901" t="s">
         <v>23</v>
@@ -49265,13 +49295,13 @@
     </row>
     <row r="902" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A902" t="s">
-        <v>2690</v>
+        <v>2689</v>
       </c>
       <c r="B902" t="s">
         <v>35</v>
       </c>
       <c r="C902" t="s">
-        <v>2691</v>
+        <v>2690</v>
       </c>
       <c r="D902" t="s">
         <v>18</v>
@@ -49286,16 +49316,16 @@
         <v>21</v>
       </c>
       <c r="H902" t="s">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="I902" t="s">
         <v>23</v>
       </c>
       <c r="J902" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
       <c r="K902" t="s">
-        <v>2686</v>
+        <v>2685</v>
       </c>
       <c r="L902" t="s">
         <v>26</v>
@@ -49309,13 +49339,13 @@
     </row>
     <row r="903" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A903" t="s">
-        <v>2693</v>
+        <v>2692</v>
       </c>
       <c r="B903" t="s">
         <v>35</v>
       </c>
       <c r="C903" t="s">
-        <v>2694</v>
+        <v>2693</v>
       </c>
       <c r="D903" t="s">
         <v>44</v>
@@ -49330,16 +49360,16 @@
         <v>21</v>
       </c>
       <c r="H903" t="s">
-        <v>2695</v>
+        <v>2694</v>
       </c>
       <c r="I903" t="s">
         <v>23</v>
       </c>
       <c r="J903" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
       <c r="K903" t="s">
-        <v>2696</v>
+        <v>2695</v>
       </c>
       <c r="L903" t="s">
         <v>44</v>
@@ -49353,13 +49383,13 @@
     </row>
     <row r="904" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A904" t="s">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="B904" t="s">
         <v>35</v>
       </c>
       <c r="C904" t="s">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="D904" t="s">
         <v>19</v>
@@ -49374,13 +49404,13 @@
         <v>21</v>
       </c>
       <c r="H904" t="s">
-        <v>2699</v>
+        <v>2698</v>
       </c>
       <c r="I904" t="s">
         <v>23</v>
       </c>
       <c r="J904" t="s">
-        <v>2700</v>
+        <v>2699</v>
       </c>
       <c r="K904" t="s">
         <v>761</v>
@@ -49397,13 +49427,13 @@
     </row>
     <row r="905" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A905" t="s">
-        <v>2701</v>
+        <v>2700</v>
       </c>
       <c r="B905" t="s">
         <v>35</v>
       </c>
       <c r="C905" t="s">
-        <v>2702</v>
+        <v>2701</v>
       </c>
       <c r="D905" t="s">
         <v>26</v>
@@ -49418,7 +49448,7 @@
         <v>21</v>
       </c>
       <c r="H905" t="s">
-        <v>2703</v>
+        <v>2702</v>
       </c>
       <c r="I905" t="s">
         <v>23</v>
@@ -49441,13 +49471,13 @@
     </row>
     <row r="906" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A906" t="s">
-        <v>2704</v>
+        <v>2703</v>
       </c>
       <c r="B906" t="s">
         <v>50</v>
       </c>
       <c r="C906" t="s">
-        <v>2705</v>
+        <v>2704</v>
       </c>
       <c r="D906" t="s">
         <v>26</v>
@@ -49462,16 +49492,16 @@
         <v>21</v>
       </c>
       <c r="H906" t="s">
-        <v>2706</v>
+        <v>2705</v>
       </c>
       <c r="I906" t="s">
         <v>23</v>
       </c>
       <c r="J906" t="s">
-        <v>2605</v>
+        <v>2604</v>
       </c>
       <c r="K906" t="s">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="L906" t="s">
         <v>26</v>
@@ -49485,13 +49515,13 @@
     </row>
     <row r="907" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A907" t="s">
-        <v>2708</v>
+        <v>2707</v>
       </c>
       <c r="B907" t="s">
         <v>50</v>
       </c>
       <c r="C907" t="s">
-        <v>2709</v>
+        <v>2708</v>
       </c>
       <c r="D907" t="s">
         <v>31</v>
@@ -49506,13 +49536,13 @@
         <v>21</v>
       </c>
       <c r="H907" t="s">
-        <v>2710</v>
+        <v>2709</v>
       </c>
       <c r="I907" t="s">
         <v>23</v>
       </c>
       <c r="J907" t="s">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="K907" t="s">
         <v>431</v>
@@ -49529,13 +49559,13 @@
     </row>
     <row r="908" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A908" t="s">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="B908" t="s">
         <v>50</v>
       </c>
       <c r="C908" t="s">
-        <v>2713</v>
+        <v>2712</v>
       </c>
       <c r="D908" t="s">
         <v>66</v>
@@ -49550,16 +49580,16 @@
         <v>21</v>
       </c>
       <c r="H908" t="s">
-        <v>2714</v>
+        <v>2713</v>
       </c>
       <c r="I908" t="s">
         <v>23</v>
       </c>
       <c r="J908" t="s">
-        <v>2700</v>
+        <v>2699</v>
       </c>
       <c r="K908" t="s">
-        <v>2894</v>
+        <v>2893</v>
       </c>
       <c r="L908" t="s">
         <v>44</v>
@@ -49573,13 +49603,13 @@
     </row>
     <row r="909" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A909" t="s">
-        <v>2715</v>
+        <v>2714</v>
       </c>
       <c r="B909" t="s">
         <v>68</v>
       </c>
       <c r="C909" t="s">
-        <v>2716</v>
+        <v>2715</v>
       </c>
       <c r="D909" t="s">
         <v>66</v>
@@ -49600,7 +49630,7 @@
         <v>23</v>
       </c>
       <c r="J909" t="s">
-        <v>2605</v>
+        <v>2604</v>
       </c>
       <c r="K909" t="s">
         <v>55</v>
@@ -49617,13 +49647,13 @@
     </row>
     <row r="910" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A910" t="s">
-        <v>2717</v>
+        <v>2716</v>
       </c>
       <c r="B910" t="s">
         <v>68</v>
       </c>
       <c r="C910" t="s">
-        <v>2718</v>
+        <v>2717</v>
       </c>
       <c r="D910" t="s">
         <v>26</v>
@@ -49638,16 +49668,16 @@
         <v>21</v>
       </c>
       <c r="H910" t="s">
-        <v>2628</v>
+        <v>2627</v>
       </c>
       <c r="I910" t="s">
         <v>23</v>
       </c>
       <c r="J910" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
       <c r="K910" t="s">
-        <v>2719</v>
+        <v>2718</v>
       </c>
       <c r="L910" t="s">
         <v>26</v>
@@ -49661,7 +49691,7 @@
     </row>
     <row r="911" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A911" t="s">
-        <v>2720</v>
+        <v>2719</v>
       </c>
       <c r="B911" t="s">
         <v>68</v>
@@ -49705,13 +49735,13 @@
     </row>
     <row r="912" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A912" t="s">
-        <v>2721</v>
+        <v>2720</v>
       </c>
       <c r="B912" t="s">
         <v>68</v>
       </c>
       <c r="C912" t="s">
-        <v>2722</v>
+        <v>2721</v>
       </c>
       <c r="D912" t="s">
         <v>19</v>
@@ -49726,7 +49756,7 @@
         <v>21</v>
       </c>
       <c r="H912" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="I912" t="s">
         <v>23</v>
@@ -49749,13 +49779,13 @@
     </row>
     <row r="913" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A913" t="s">
-        <v>2723</v>
+        <v>2722</v>
       </c>
       <c r="B913" t="s">
         <v>68</v>
       </c>
       <c r="C913" t="s">
-        <v>2724</v>
+        <v>2723</v>
       </c>
       <c r="D913" t="s">
         <v>44</v>
@@ -49770,7 +49800,7 @@
         <v>21</v>
       </c>
       <c r="H913" t="s">
-        <v>2725</v>
+        <v>2724</v>
       </c>
       <c r="I913" t="s">
         <v>23</v>
@@ -49793,13 +49823,13 @@
     </row>
     <row r="914" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A914" t="s">
-        <v>2726</v>
+        <v>2725</v>
       </c>
       <c r="B914" t="s">
         <v>68</v>
       </c>
       <c r="C914" t="s">
-        <v>2727</v>
+        <v>2726</v>
       </c>
       <c r="D914" t="s">
         <v>44</v>
@@ -49823,7 +49853,7 @@
         <v>1811</v>
       </c>
       <c r="K914" t="s">
-        <v>2728</v>
+        <v>2727</v>
       </c>
       <c r="L914" t="s">
         <v>70</v>
@@ -49837,7 +49867,7 @@
     </row>
     <row r="915" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A915" t="s">
-        <v>2729</v>
+        <v>2728</v>
       </c>
       <c r="B915" t="s">
         <v>35</v>
@@ -49858,13 +49888,13 @@
         <v>223</v>
       </c>
       <c r="H915" t="s">
+        <v>2729</v>
+      </c>
+      <c r="I915" t="s">
+        <v>55</v>
+      </c>
+      <c r="J915" t="s">
         <v>2730</v>
-      </c>
-      <c r="I915" t="s">
-        <v>55</v>
-      </c>
-      <c r="J915" t="s">
-        <v>2731</v>
       </c>
       <c r="K915" t="s">
         <v>55</v>
@@ -49881,13 +49911,13 @@
     </row>
     <row r="916" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A916" t="s">
-        <v>2732</v>
+        <v>2731</v>
       </c>
       <c r="B916" t="s">
         <v>50</v>
       </c>
       <c r="C916" t="s">
-        <v>2733</v>
+        <v>2732</v>
       </c>
       <c r="D916" t="s">
         <v>26</v>
@@ -49902,13 +49932,13 @@
         <v>223</v>
       </c>
       <c r="H916" t="s">
-        <v>2734</v>
+        <v>2733</v>
       </c>
       <c r="I916" t="s">
         <v>55</v>
       </c>
       <c r="J916" t="s">
-        <v>2731</v>
+        <v>2730</v>
       </c>
       <c r="K916" t="s">
         <v>55</v>
@@ -49925,7 +49955,7 @@
     </row>
     <row r="917" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A917" t="s">
-        <v>2735</v>
+        <v>2734</v>
       </c>
       <c r="B917" t="s">
         <v>50</v>
@@ -49946,7 +49976,7 @@
         <v>223</v>
       </c>
       <c r="H917" t="s">
-        <v>2736</v>
+        <v>2735</v>
       </c>
       <c r="I917" t="s">
         <v>55</v>
@@ -49969,13 +49999,13 @@
     </row>
     <row r="918" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A918" t="s">
-        <v>2737</v>
+        <v>2736</v>
       </c>
       <c r="B918" t="s">
         <v>68</v>
       </c>
       <c r="C918" t="s">
-        <v>2738</v>
+        <v>2737</v>
       </c>
       <c r="D918" t="s">
         <v>44</v>
@@ -49990,7 +50020,7 @@
         <v>223</v>
       </c>
       <c r="H918" t="s">
-        <v>2739</v>
+        <v>2738</v>
       </c>
       <c r="I918" t="s">
         <v>55</v>
@@ -50013,7 +50043,7 @@
     </row>
     <row r="919" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A919" t="s">
-        <v>2740</v>
+        <v>2739</v>
       </c>
       <c r="B919" t="s">
         <v>35</v>
@@ -50034,13 +50064,13 @@
         <v>223</v>
       </c>
       <c r="H919" t="s">
+        <v>2740</v>
+      </c>
+      <c r="I919" t="s">
+        <v>55</v>
+      </c>
+      <c r="J919" t="s">
         <v>2741</v>
-      </c>
-      <c r="I919" t="s">
-        <v>55</v>
-      </c>
-      <c r="J919" t="s">
-        <v>2742</v>
       </c>
       <c r="K919" t="s">
         <v>55</v>
@@ -50057,13 +50087,13 @@
     </row>
     <row r="920" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A920" t="s">
-        <v>2743</v>
+        <v>2742</v>
       </c>
       <c r="B920" t="s">
         <v>50</v>
       </c>
       <c r="C920" t="s">
-        <v>2744</v>
+        <v>2743</v>
       </c>
       <c r="D920" t="s">
         <v>44</v>
@@ -50078,7 +50108,7 @@
         <v>223</v>
       </c>
       <c r="H920" t="s">
-        <v>2745</v>
+        <v>2744</v>
       </c>
       <c r="I920" t="s">
         <v>55</v>
@@ -50101,13 +50131,13 @@
     </row>
     <row r="921" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A921" t="s">
-        <v>2746</v>
+        <v>2745</v>
       </c>
       <c r="B921" t="s">
         <v>50</v>
       </c>
       <c r="C921" t="s">
-        <v>2747</v>
+        <v>2746</v>
       </c>
       <c r="D921" t="s">
         <v>44</v>
@@ -50122,7 +50152,7 @@
         <v>223</v>
       </c>
       <c r="H921" t="s">
-        <v>2748</v>
+        <v>2747</v>
       </c>
       <c r="I921" t="s">
         <v>55</v>
@@ -50145,13 +50175,13 @@
     </row>
     <row r="922" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A922" t="s">
-        <v>2749</v>
+        <v>2748</v>
       </c>
       <c r="B922" t="s">
         <v>68</v>
       </c>
       <c r="C922" t="s">
-        <v>2750</v>
+        <v>2749</v>
       </c>
       <c r="D922" t="s">
         <v>19</v>
@@ -50166,13 +50196,13 @@
         <v>223</v>
       </c>
       <c r="H922" t="s">
-        <v>2751</v>
+        <v>2750</v>
       </c>
       <c r="I922" t="s">
         <v>55</v>
       </c>
       <c r="J922" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="K922" t="s">
         <v>55</v>
@@ -50189,13 +50219,13 @@
     </row>
     <row r="923" spans="1:14" ht="29" x14ac:dyDescent="0.3">
       <c r="A923" t="s">
-        <v>2752</v>
+        <v>2751</v>
       </c>
       <c r="B923" t="s">
         <v>16</v>
       </c>
       <c r="C923" t="s">
-        <v>2753</v>
+        <v>2752</v>
       </c>
       <c r="D923" t="s">
         <v>18</v>
@@ -50210,13 +50240,13 @@
         <v>223</v>
       </c>
       <c r="H923" s="1" t="s">
-        <v>2893</v>
+        <v>2892</v>
       </c>
       <c r="I923" t="s">
         <v>55</v>
       </c>
       <c r="J923" t="s">
-        <v>2754</v>
+        <v>2753</v>
       </c>
       <c r="K923" t="s">
         <v>55</v>
@@ -50233,13 +50263,13 @@
     </row>
     <row r="924" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A924" t="s">
-        <v>2755</v>
+        <v>2754</v>
       </c>
       <c r="B924" t="s">
         <v>35</v>
       </c>
       <c r="C924" t="s">
-        <v>2756</v>
+        <v>2755</v>
       </c>
       <c r="D924" t="s">
         <v>44</v>
@@ -50254,13 +50284,13 @@
         <v>223</v>
       </c>
       <c r="H924" t="s">
+        <v>2756</v>
+      </c>
+      <c r="I924" t="s">
+        <v>55</v>
+      </c>
+      <c r="J924" t="s">
         <v>2757</v>
-      </c>
-      <c r="I924" t="s">
-        <v>55</v>
-      </c>
-      <c r="J924" t="s">
-        <v>2758</v>
       </c>
       <c r="K924" t="s">
         <v>55</v>
@@ -50277,13 +50307,13 @@
     </row>
     <row r="925" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A925" t="s">
-        <v>2759</v>
+        <v>2758</v>
       </c>
       <c r="B925" t="s">
         <v>50</v>
       </c>
       <c r="C925" t="s">
-        <v>2760</v>
+        <v>2759</v>
       </c>
       <c r="D925" t="s">
         <v>44</v>
@@ -50298,13 +50328,13 @@
         <v>223</v>
       </c>
       <c r="H925" t="s">
-        <v>2761</v>
+        <v>2760</v>
       </c>
       <c r="I925" t="s">
         <v>55</v>
       </c>
       <c r="J925" t="s">
-        <v>2758</v>
+        <v>2757</v>
       </c>
       <c r="K925" t="s">
         <v>55</v>
@@ -50321,13 +50351,13 @@
     </row>
     <row r="926" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A926" t="s">
-        <v>2762</v>
+        <v>2761</v>
       </c>
       <c r="B926" t="s">
         <v>68</v>
       </c>
       <c r="C926" t="s">
-        <v>2763</v>
+        <v>2762</v>
       </c>
       <c r="D926" t="s">
         <v>44</v>
@@ -50342,13 +50372,13 @@
         <v>223</v>
       </c>
       <c r="H926" t="s">
-        <v>2764</v>
+        <v>2763</v>
       </c>
       <c r="I926" t="s">
         <v>55</v>
       </c>
       <c r="J926" t="s">
-        <v>2758</v>
+        <v>2757</v>
       </c>
       <c r="K926" t="s">
         <v>55</v>
@@ -50365,7 +50395,7 @@
     </row>
     <row r="927" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A927" t="s">
-        <v>2765</v>
+        <v>2764</v>
       </c>
       <c r="B927" t="s">
         <v>35</v>
@@ -50386,7 +50416,7 @@
         <v>223</v>
       </c>
       <c r="H927" t="s">
-        <v>2766</v>
+        <v>2765</v>
       </c>
       <c r="I927" t="s">
         <v>55</v>
@@ -50409,13 +50439,13 @@
     </row>
     <row r="928" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A928" t="s">
-        <v>2767</v>
+        <v>2766</v>
       </c>
       <c r="B928" t="s">
         <v>50</v>
       </c>
       <c r="C928" t="s">
-        <v>2768</v>
+        <v>2767</v>
       </c>
       <c r="D928" t="s">
         <v>44</v>
@@ -50430,7 +50460,7 @@
         <v>223</v>
       </c>
       <c r="H928" t="s">
-        <v>2769</v>
+        <v>2768</v>
       </c>
       <c r="I928" t="s">
         <v>55</v>
@@ -50453,13 +50483,13 @@
     </row>
     <row r="929" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A929" t="s">
-        <v>2770</v>
+        <v>2769</v>
       </c>
       <c r="B929" t="s">
         <v>68</v>
       </c>
       <c r="C929" t="s">
-        <v>2771</v>
+        <v>2770</v>
       </c>
       <c r="D929" t="s">
         <v>26</v>
@@ -50474,7 +50504,7 @@
         <v>223</v>
       </c>
       <c r="H929" t="s">
-        <v>2772</v>
+        <v>2771</v>
       </c>
       <c r="I929" t="s">
         <v>55</v>
@@ -50497,13 +50527,13 @@
     </row>
     <row r="930" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A930" t="s">
-        <v>2773</v>
+        <v>2772</v>
       </c>
       <c r="B930" t="s">
         <v>68</v>
       </c>
       <c r="C930" t="s">
-        <v>2774</v>
+        <v>2773</v>
       </c>
       <c r="D930" t="s">
         <v>44</v>
@@ -50518,7 +50548,7 @@
         <v>223</v>
       </c>
       <c r="H930" t="s">
-        <v>2775</v>
+        <v>2774</v>
       </c>
       <c r="I930" t="s">
         <v>55</v>
@@ -50541,13 +50571,13 @@
     </row>
     <row r="931" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A931" t="s">
-        <v>2776</v>
+        <v>2775</v>
       </c>
       <c r="B931" t="s">
         <v>35</v>
       </c>
       <c r="C931" t="s">
-        <v>2777</v>
+        <v>2776</v>
       </c>
       <c r="D931" t="s">
         <v>26</v>
@@ -50562,13 +50592,13 @@
         <v>223</v>
       </c>
       <c r="H931" t="s">
+        <v>2777</v>
+      </c>
+      <c r="I931" t="s">
+        <v>55</v>
+      </c>
+      <c r="J931" t="s">
         <v>2778</v>
-      </c>
-      <c r="I931" t="s">
-        <v>55</v>
-      </c>
-      <c r="J931" t="s">
-        <v>2779</v>
       </c>
       <c r="K931" t="s">
         <v>55</v>
@@ -50585,7 +50615,7 @@
     </row>
     <row r="932" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A932" t="s">
-        <v>2780</v>
+        <v>2779</v>
       </c>
       <c r="B932" t="s">
         <v>35</v>
@@ -50606,13 +50636,13 @@
         <v>223</v>
       </c>
       <c r="H932" t="s">
+        <v>2780</v>
+      </c>
+      <c r="I932" t="s">
+        <v>55</v>
+      </c>
+      <c r="J932" t="s">
         <v>2781</v>
-      </c>
-      <c r="I932" t="s">
-        <v>55</v>
-      </c>
-      <c r="J932" t="s">
-        <v>2782</v>
       </c>
       <c r="K932" t="s">
         <v>55</v>
@@ -50629,13 +50659,13 @@
     </row>
     <row r="933" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A933" t="s">
-        <v>2783</v>
+        <v>2782</v>
       </c>
       <c r="B933" t="s">
         <v>50</v>
       </c>
       <c r="C933" t="s">
-        <v>2784</v>
+        <v>2783</v>
       </c>
       <c r="D933" t="s">
         <v>26</v>
@@ -50650,13 +50680,13 @@
         <v>223</v>
       </c>
       <c r="H933" t="s">
-        <v>2785</v>
+        <v>2784</v>
       </c>
       <c r="I933" t="s">
         <v>55</v>
       </c>
       <c r="J933" t="s">
-        <v>2782</v>
+        <v>2781</v>
       </c>
       <c r="K933" t="s">
         <v>55</v>
@@ -50673,13 +50703,13 @@
     </row>
     <row r="934" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A934" t="s">
-        <v>2786</v>
+        <v>2785</v>
       </c>
       <c r="B934" t="s">
         <v>50</v>
       </c>
       <c r="C934" t="s">
-        <v>2787</v>
+        <v>2786</v>
       </c>
       <c r="D934" t="s">
         <v>26</v>
@@ -50694,13 +50724,13 @@
         <v>223</v>
       </c>
       <c r="H934" t="s">
-        <v>2788</v>
+        <v>2787</v>
       </c>
       <c r="I934" t="s">
         <v>55</v>
       </c>
       <c r="J934" t="s">
-        <v>2782</v>
+        <v>2781</v>
       </c>
       <c r="K934" t="s">
         <v>55</v>
@@ -50717,13 +50747,13 @@
     </row>
     <row r="935" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A935" t="s">
-        <v>2789</v>
+        <v>2788</v>
       </c>
       <c r="B935" t="s">
         <v>68</v>
       </c>
       <c r="C935" t="s">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="D935" t="s">
         <v>44</v>
@@ -50738,7 +50768,7 @@
         <v>223</v>
       </c>
       <c r="H935" t="s">
-        <v>2791</v>
+        <v>2790</v>
       </c>
       <c r="I935" t="s">
         <v>55</v>
@@ -50761,13 +50791,13 @@
     </row>
     <row r="936" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A936" t="s">
-        <v>2792</v>
+        <v>2791</v>
       </c>
       <c r="B936" t="s">
         <v>35</v>
       </c>
       <c r="C936" t="s">
-        <v>2793</v>
+        <v>2792</v>
       </c>
       <c r="D936" t="s">
         <v>19</v>
@@ -50782,7 +50812,7 @@
         <v>265</v>
       </c>
       <c r="H936" t="s">
-        <v>2794</v>
+        <v>2793</v>
       </c>
       <c r="I936" t="s">
         <v>55</v>
@@ -50805,13 +50835,13 @@
     </row>
     <row r="937" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A937" t="s">
-        <v>2795</v>
+        <v>2794</v>
       </c>
       <c r="B937" t="s">
         <v>50</v>
       </c>
       <c r="C937" t="s">
-        <v>2796</v>
+        <v>2795</v>
       </c>
       <c r="D937" t="s">
         <v>26</v>
@@ -50826,7 +50856,7 @@
         <v>265</v>
       </c>
       <c r="H937" t="s">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="I937" t="s">
         <v>55</v>
@@ -50849,13 +50879,13 @@
     </row>
     <row r="938" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A938" t="s">
-        <v>2798</v>
+        <v>2797</v>
       </c>
       <c r="B938" t="s">
         <v>68</v>
       </c>
       <c r="C938" t="s">
-        <v>2799</v>
+        <v>2798</v>
       </c>
       <c r="D938" t="s">
         <v>44</v>
@@ -50870,7 +50900,7 @@
         <v>265</v>
       </c>
       <c r="H938" t="s">
-        <v>2800</v>
+        <v>2799</v>
       </c>
       <c r="I938" t="s">
         <v>55</v>
@@ -50893,13 +50923,13 @@
     </row>
     <row r="939" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A939" t="s">
-        <v>2801</v>
+        <v>2800</v>
       </c>
       <c r="B939" t="s">
         <v>68</v>
       </c>
       <c r="C939" t="s">
-        <v>2802</v>
+        <v>2801</v>
       </c>
       <c r="D939" t="s">
         <v>66</v>
@@ -50914,7 +50944,7 @@
         <v>265</v>
       </c>
       <c r="H939" t="s">
-        <v>2803</v>
+        <v>2802</v>
       </c>
       <c r="I939" t="s">
         <v>55</v>
@@ -50937,13 +50967,13 @@
     </row>
     <row r="940" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A940" t="s">
-        <v>2804</v>
+        <v>2803</v>
       </c>
       <c r="B940" t="s">
         <v>35</v>
       </c>
       <c r="C940" t="s">
-        <v>2805</v>
+        <v>2804</v>
       </c>
       <c r="D940" t="s">
         <v>44</v>
@@ -50958,7 +50988,7 @@
         <v>265</v>
       </c>
       <c r="H940" t="s">
-        <v>2806</v>
+        <v>2805</v>
       </c>
       <c r="I940" t="s">
         <v>55</v>
@@ -50981,19 +51011,19 @@
     </row>
     <row r="941" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A941" t="s">
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="B941" t="s">
         <v>50</v>
       </c>
       <c r="C941" t="s">
+        <v>2807</v>
+      </c>
+      <c r="D941" t="s">
         <v>2808</v>
       </c>
-      <c r="D941" t="s">
-        <v>2809</v>
-      </c>
       <c r="E941" t="s">
-        <v>2809</v>
+        <v>2808</v>
       </c>
       <c r="F941" t="s">
         <v>101</v>
@@ -51002,7 +51032,7 @@
         <v>265</v>
       </c>
       <c r="H941" t="s">
-        <v>2810</v>
+        <v>2809</v>
       </c>
       <c r="I941" t="s">
         <v>55</v>
@@ -51025,13 +51055,13 @@
     </row>
     <row r="942" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A942" t="s">
-        <v>2811</v>
+        <v>2810</v>
       </c>
       <c r="B942" t="s">
         <v>68</v>
       </c>
       <c r="C942" t="s">
-        <v>2812</v>
+        <v>2811</v>
       </c>
       <c r="D942" t="s">
         <v>44</v>
@@ -51046,7 +51076,7 @@
         <v>265</v>
       </c>
       <c r="H942" t="s">
-        <v>2813</v>
+        <v>2812</v>
       </c>
       <c r="I942" t="s">
         <v>55</v>
@@ -51069,13 +51099,13 @@
     </row>
     <row r="943" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A943" t="s">
-        <v>2814</v>
+        <v>2813</v>
       </c>
       <c r="B943" t="s">
         <v>68</v>
       </c>
       <c r="C943" t="s">
-        <v>2815</v>
+        <v>2814</v>
       </c>
       <c r="D943" t="s">
         <v>44</v>
@@ -51090,7 +51120,7 @@
         <v>265</v>
       </c>
       <c r="H943" t="s">
-        <v>2816</v>
+        <v>2815</v>
       </c>
       <c r="I943" t="s">
         <v>55</v>
@@ -51113,13 +51143,13 @@
     </row>
     <row r="944" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A944" t="s">
-        <v>2817</v>
+        <v>2816</v>
       </c>
       <c r="B944" t="s">
         <v>35</v>
       </c>
       <c r="C944" t="s">
-        <v>2818</v>
+        <v>2817</v>
       </c>
       <c r="D944" t="s">
         <v>26</v>
@@ -51134,13 +51164,13 @@
         <v>265</v>
       </c>
       <c r="H944" t="s">
+        <v>2818</v>
+      </c>
+      <c r="I944" t="s">
+        <v>55</v>
+      </c>
+      <c r="J944" t="s">
         <v>2819</v>
-      </c>
-      <c r="I944" t="s">
-        <v>55</v>
-      </c>
-      <c r="J944" t="s">
-        <v>2820</v>
       </c>
       <c r="K944" t="s">
         <v>55</v>
@@ -51157,13 +51187,13 @@
     </row>
     <row r="945" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A945" t="s">
-        <v>2821</v>
+        <v>2820</v>
       </c>
       <c r="B945" t="s">
         <v>50</v>
       </c>
       <c r="C945" t="s">
-        <v>2822</v>
+        <v>2821</v>
       </c>
       <c r="D945" t="s">
         <v>70</v>
@@ -51178,7 +51208,7 @@
         <v>265</v>
       </c>
       <c r="H945" t="s">
-        <v>2823</v>
+        <v>2822</v>
       </c>
       <c r="I945" t="s">
         <v>55</v>
@@ -51201,13 +51231,13 @@
     </row>
     <row r="946" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A946" t="s">
-        <v>2824</v>
+        <v>2823</v>
       </c>
       <c r="B946" t="s">
         <v>68</v>
       </c>
       <c r="C946" t="s">
-        <v>2825</v>
+        <v>2824</v>
       </c>
       <c r="D946" t="s">
         <v>26</v>
@@ -51222,13 +51252,13 @@
         <v>265</v>
       </c>
       <c r="H946" t="s">
+        <v>2825</v>
+      </c>
+      <c r="I946" t="s">
+        <v>55</v>
+      </c>
+      <c r="J946" t="s">
         <v>2826</v>
-      </c>
-      <c r="I946" t="s">
-        <v>55</v>
-      </c>
-      <c r="J946" t="s">
-        <v>2827</v>
       </c>
       <c r="K946" t="s">
         <v>55</v>
@@ -51245,13 +51275,13 @@
     </row>
     <row r="947" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A947" t="s">
-        <v>2828</v>
+        <v>2827</v>
       </c>
       <c r="B947" t="s">
         <v>68</v>
       </c>
       <c r="C947" t="s">
-        <v>2829</v>
+        <v>2828</v>
       </c>
       <c r="D947" t="s">
         <v>44</v>
@@ -51266,13 +51296,13 @@
         <v>265</v>
       </c>
       <c r="H947" t="s">
-        <v>2830</v>
+        <v>2829</v>
       </c>
       <c r="I947" t="s">
         <v>55</v>
       </c>
       <c r="J947" t="s">
-        <v>2827</v>
+        <v>2826</v>
       </c>
       <c r="K947" t="s">
         <v>55</v>
@@ -51289,13 +51319,13 @@
     </row>
     <row r="948" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A948" t="s">
-        <v>2831</v>
+        <v>2830</v>
       </c>
       <c r="B948" t="s">
         <v>35</v>
       </c>
       <c r="C948" t="s">
-        <v>2832</v>
+        <v>2831</v>
       </c>
       <c r="D948" t="s">
         <v>18</v>
@@ -51310,7 +51340,7 @@
         <v>265</v>
       </c>
       <c r="H948" t="s">
-        <v>2833</v>
+        <v>2832</v>
       </c>
       <c r="I948" t="s">
         <v>55</v>
@@ -51333,13 +51363,13 @@
     </row>
     <row r="949" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A949" t="s">
-        <v>2834</v>
+        <v>2833</v>
       </c>
       <c r="B949" t="s">
         <v>50</v>
       </c>
       <c r="C949" t="s">
-        <v>2835</v>
+        <v>2834</v>
       </c>
       <c r="D949" t="s">
         <v>18</v>
@@ -51354,7 +51384,7 @@
         <v>265</v>
       </c>
       <c r="H949" t="s">
-        <v>2836</v>
+        <v>2835</v>
       </c>
       <c r="I949" t="s">
         <v>55</v>
@@ -51377,13 +51407,13 @@
     </row>
     <row r="950" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A950" t="s">
-        <v>2837</v>
+        <v>2836</v>
       </c>
       <c r="B950" t="s">
         <v>68</v>
       </c>
       <c r="C950" t="s">
-        <v>2838</v>
+        <v>2837</v>
       </c>
       <c r="D950" t="s">
         <v>66</v>
@@ -51398,7 +51428,7 @@
         <v>265</v>
       </c>
       <c r="H950" t="s">
-        <v>2839</v>
+        <v>2838</v>
       </c>
       <c r="I950" t="s">
         <v>55</v>
@@ -51421,13 +51451,13 @@
     </row>
     <row r="951" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A951" t="s">
-        <v>2840</v>
+        <v>2839</v>
       </c>
       <c r="B951" t="s">
         <v>68</v>
       </c>
       <c r="C951" t="s">
-        <v>2841</v>
+        <v>2840</v>
       </c>
       <c r="D951" t="s">
         <v>44</v>
@@ -51442,7 +51472,7 @@
         <v>265</v>
       </c>
       <c r="H951" t="s">
-        <v>2842</v>
+        <v>2841</v>
       </c>
       <c r="I951" t="s">
         <v>55</v>
@@ -51465,13 +51495,13 @@
     </row>
     <row r="952" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A952" t="s">
-        <v>2843</v>
+        <v>2842</v>
       </c>
       <c r="B952" t="s">
         <v>50</v>
       </c>
       <c r="C952" t="s">
-        <v>2844</v>
+        <v>2843</v>
       </c>
       <c r="D952" t="s">
         <v>44</v>
@@ -51486,7 +51516,7 @@
         <v>265</v>
       </c>
       <c r="H952" t="s">
-        <v>2845</v>
+        <v>2844</v>
       </c>
       <c r="I952" t="s">
         <v>55</v>
@@ -51509,13 +51539,13 @@
     </row>
     <row r="953" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A953" t="s">
-        <v>2846</v>
+        <v>2845</v>
       </c>
       <c r="B953" t="s">
         <v>35</v>
       </c>
       <c r="C953" t="s">
-        <v>2847</v>
+        <v>2846</v>
       </c>
       <c r="D953" t="s">
         <v>19</v>
@@ -51530,13 +51560,13 @@
         <v>265</v>
       </c>
       <c r="H953" t="s">
-        <v>2848</v>
+        <v>2847</v>
       </c>
       <c r="I953" t="s">
         <v>55</v>
       </c>
       <c r="J953" t="s">
-        <v>2700</v>
+        <v>2699</v>
       </c>
       <c r="K953" t="s">
         <v>55</v>
@@ -51553,13 +51583,13 @@
     </row>
     <row r="954" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A954" t="s">
-        <v>2849</v>
+        <v>2848</v>
       </c>
       <c r="B954" t="s">
         <v>50</v>
       </c>
       <c r="C954" t="s">
-        <v>2850</v>
+        <v>2849</v>
       </c>
       <c r="D954" t="s">
         <v>26</v>
@@ -51574,13 +51604,13 @@
         <v>265</v>
       </c>
       <c r="H954" t="s">
+        <v>2850</v>
+      </c>
+      <c r="I954" t="s">
+        <v>55</v>
+      </c>
+      <c r="J954" t="s">
         <v>2851</v>
-      </c>
-      <c r="I954" t="s">
-        <v>55</v>
-      </c>
-      <c r="J954" t="s">
-        <v>2852</v>
       </c>
       <c r="K954" t="s">
         <v>55</v>
@@ -51597,13 +51627,13 @@
     </row>
     <row r="955" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A955" t="s">
-        <v>2853</v>
+        <v>2852</v>
       </c>
       <c r="B955" t="s">
         <v>68</v>
       </c>
       <c r="C955" t="s">
-        <v>2854</v>
+        <v>2853</v>
       </c>
       <c r="D955" t="s">
         <v>44</v>
@@ -51618,13 +51648,13 @@
         <v>265</v>
       </c>
       <c r="H955" t="s">
-        <v>2855</v>
+        <v>2854</v>
       </c>
       <c r="I955" t="s">
         <v>55</v>
       </c>
       <c r="J955" t="s">
-        <v>2827</v>
+        <v>2826</v>
       </c>
       <c r="K955" t="s">
         <v>55</v>
@@ -51641,13 +51671,13 @@
     </row>
     <row r="956" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A956" t="s">
-        <v>2856</v>
+        <v>2855</v>
       </c>
       <c r="B956" t="s">
         <v>68</v>
       </c>
       <c r="C956" t="s">
-        <v>2857</v>
+        <v>2856</v>
       </c>
       <c r="D956" t="s">
         <v>26</v>
@@ -51662,13 +51692,13 @@
         <v>265</v>
       </c>
       <c r="H956" t="s">
-        <v>2858</v>
+        <v>2857</v>
       </c>
       <c r="I956" t="s">
         <v>55</v>
       </c>
       <c r="J956" t="s">
-        <v>2827</v>
+        <v>2826</v>
       </c>
       <c r="K956" t="s">
         <v>55</v>
@@ -51685,7 +51715,7 @@
     </row>
     <row r="957" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A957" t="s">
-        <v>2859</v>
+        <v>2858</v>
       </c>
       <c r="B957" t="s">
         <v>50</v>
@@ -51706,13 +51736,13 @@
         <v>302</v>
       </c>
       <c r="H957" t="s">
-        <v>2860</v>
+        <v>2859</v>
       </c>
       <c r="I957" t="s">
         <v>23</v>
       </c>
       <c r="J957" t="s">
-        <v>2861</v>
+        <v>2860</v>
       </c>
       <c r="K957" t="s">
         <v>55</v>
@@ -51729,13 +51759,13 @@
     </row>
     <row r="958" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A958" t="s">
-        <v>2862</v>
+        <v>2861</v>
       </c>
       <c r="B958" t="s">
         <v>68</v>
       </c>
       <c r="C958" t="s">
-        <v>2863</v>
+        <v>2862</v>
       </c>
       <c r="D958" t="s">
         <v>66</v>
@@ -51750,7 +51780,7 @@
         <v>302</v>
       </c>
       <c r="H958" t="s">
-        <v>2864</v>
+        <v>2863</v>
       </c>
       <c r="I958" t="s">
         <v>23</v>
@@ -51773,13 +51803,13 @@
     </row>
     <row r="959" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A959" t="s">
-        <v>2865</v>
+        <v>2864</v>
       </c>
       <c r="B959" t="s">
         <v>50</v>
       </c>
       <c r="C959" t="s">
-        <v>2866</v>
+        <v>2865</v>
       </c>
       <c r="D959" t="s">
         <v>44</v>
@@ -51794,13 +51824,13 @@
         <v>302</v>
       </c>
       <c r="H959" t="s">
-        <v>2867</v>
+        <v>2866</v>
       </c>
       <c r="I959" t="s">
         <v>38</v>
       </c>
       <c r="J959" t="s">
-        <v>2868</v>
+        <v>2867</v>
       </c>
       <c r="K959" t="s">
         <v>55</v>
@@ -51817,13 +51847,13 @@
     </row>
     <row r="960" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A960" t="s">
-        <v>2869</v>
+        <v>2868</v>
       </c>
       <c r="B960" t="s">
         <v>68</v>
       </c>
       <c r="C960" t="s">
-        <v>2870</v>
+        <v>2869</v>
       </c>
       <c r="D960" t="s">
         <v>18</v>
@@ -51838,13 +51868,13 @@
         <v>302</v>
       </c>
       <c r="H960" t="s">
-        <v>2871</v>
+        <v>2870</v>
       </c>
       <c r="I960" t="s">
         <v>38</v>
       </c>
       <c r="J960" t="s">
-        <v>2872</v>
+        <v>2871</v>
       </c>
       <c r="K960" t="s">
         <v>55</v>
@@ -51861,13 +51891,13 @@
     </row>
     <row r="961" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A961" t="s">
-        <v>2873</v>
+        <v>2872</v>
       </c>
       <c r="B961" t="s">
         <v>50</v>
       </c>
       <c r="C961" t="s">
-        <v>2874</v>
+        <v>2873</v>
       </c>
       <c r="D961" t="s">
         <v>66</v>
@@ -51882,13 +51912,13 @@
         <v>302</v>
       </c>
       <c r="H961" t="s">
-        <v>2875</v>
+        <v>2874</v>
       </c>
       <c r="I961" t="s">
         <v>38</v>
       </c>
       <c r="J961" t="s">
-        <v>2876</v>
+        <v>2875</v>
       </c>
       <c r="K961" t="s">
         <v>55</v>
@@ -51905,13 +51935,13 @@
     </row>
     <row r="962" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A962" t="s">
-        <v>2877</v>
+        <v>2876</v>
       </c>
       <c r="B962" t="s">
         <v>68</v>
       </c>
       <c r="C962" t="s">
-        <v>2878</v>
+        <v>2877</v>
       </c>
       <c r="D962" t="s">
         <v>44</v>
@@ -51926,13 +51956,13 @@
         <v>302</v>
       </c>
       <c r="H962" t="s">
-        <v>2879</v>
+        <v>2878</v>
       </c>
       <c r="I962" t="s">
         <v>80</v>
       </c>
       <c r="J962" t="s">
-        <v>2880</v>
+        <v>2879</v>
       </c>
       <c r="K962" t="s">
         <v>55</v>
@@ -51949,13 +51979,13 @@
     </row>
     <row r="963" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A963" t="s">
-        <v>2881</v>
+        <v>2880</v>
       </c>
       <c r="B963" t="s">
         <v>35</v>
       </c>
       <c r="C963" t="s">
-        <v>2882</v>
+        <v>2881</v>
       </c>
       <c r="D963" t="s">
         <v>26</v>
@@ -51970,7 +52000,7 @@
         <v>302</v>
       </c>
       <c r="H963" t="s">
-        <v>2883</v>
+        <v>2882</v>
       </c>
       <c r="I963" t="s">
         <v>38</v>
@@ -51993,13 +52023,13 @@
     </row>
     <row r="964" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A964" t="s">
-        <v>2884</v>
+        <v>2883</v>
       </c>
       <c r="B964" t="s">
         <v>68</v>
       </c>
       <c r="C964" t="s">
-        <v>2885</v>
+        <v>2884</v>
       </c>
       <c r="D964" t="s">
         <v>66</v>
@@ -52014,13 +52044,13 @@
         <v>302</v>
       </c>
       <c r="H964" t="s">
-        <v>2886</v>
+        <v>2885</v>
       </c>
       <c r="I964" t="s">
         <v>80</v>
       </c>
       <c r="J964" t="s">
-        <v>2887</v>
+        <v>2886</v>
       </c>
       <c r="K964" t="s">
         <v>55</v>
@@ -52037,13 +52067,13 @@
     </row>
     <row r="965" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A965" t="s">
-        <v>2888</v>
+        <v>2887</v>
       </c>
       <c r="B965" t="s">
         <v>68</v>
       </c>
       <c r="C965" t="s">
-        <v>2889</v>
+        <v>2888</v>
       </c>
       <c r="D965" t="s">
         <v>55</v>
@@ -52058,13 +52088,13 @@
         <v>2456</v>
       </c>
       <c r="H965" t="s">
-        <v>2890</v>
+        <v>2889</v>
       </c>
       <c r="I965" t="s">
         <v>55</v>
       </c>
       <c r="J965" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="K965" t="s">
         <v>55</v>
@@ -52081,13 +52111,13 @@
     </row>
     <row r="966" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A966" t="s">
-        <v>2891</v>
+        <v>2890</v>
       </c>
       <c r="B966" t="s">
         <v>68</v>
       </c>
       <c r="C966" t="s">
-        <v>2892</v>
+        <v>2891</v>
       </c>
       <c r="D966" t="s">
         <v>55</v>

</xml_diff>